<commit_message>
staged codes for updated measures & gravity model
</commit_message>
<xml_diff>
--- a/poi/category-list-purpose-annotated.xlsx
+++ b/poi/category-list-purpose-annotated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mario/github/google-poi-japan/poi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1B098EF-C5E7-F64A-871D-B884BFFC04BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0B436CC-01D7-D74F-A7AA-802926125762}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="120">
   <si>
     <t>primary</t>
   </si>
@@ -373,6 +373,26 @@
   </si>
   <si>
     <t>visiting</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>consuming</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>working</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>working/visiting</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>learning</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>learning/visiting</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -806,14 +826,24 @@
       <c r="C2" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
+      <c r="D2" s="2">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2">
+        <v>2</v>
+      </c>
+      <c r="F2" s="2">
+        <v>2</v>
+      </c>
+      <c r="G2" s="2">
+        <v>2</v>
+      </c>
       <c r="H2" s="2">
-        <v>1</v>
-      </c>
-      <c r="I2" s="2"/>
+        <v>2</v>
+      </c>
+      <c r="I2" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="3" spans="1:9" ht="15">
       <c r="A3" s="2" t="s">
@@ -825,14 +855,24 @@
       <c r="C3" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
+      <c r="D3" s="2">
+        <v>2</v>
+      </c>
+      <c r="E3" s="2">
+        <v>2</v>
+      </c>
+      <c r="F3" s="2">
+        <v>2</v>
+      </c>
       <c r="G3" s="2">
-        <v>1</v>
-      </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
+        <v>2</v>
+      </c>
+      <c r="H3" s="2">
+        <v>2</v>
+      </c>
+      <c r="I3" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" spans="1:9" ht="15">
       <c r="A4" s="2" t="s">
@@ -844,18 +884,24 @@
       <c r="C4" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D4" s="2"/>
+      <c r="D4" s="2">
+        <v>0</v>
+      </c>
       <c r="E4" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4" s="2">
-        <v>1</v>
-      </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
+        <v>2</v>
+      </c>
+      <c r="H4" s="2">
+        <v>0</v>
+      </c>
+      <c r="I4" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" spans="1:9" ht="15">
       <c r="A5" s="2" t="s">
@@ -868,15 +914,23 @@
         <v>113</v>
       </c>
       <c r="D5" s="2">
-        <v>1</v>
-      </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
+        <v>2</v>
+      </c>
+      <c r="E5" s="2">
+        <v>0</v>
+      </c>
+      <c r="F5" s="2">
+        <v>1</v>
+      </c>
+      <c r="G5" s="2">
+        <v>1</v>
+      </c>
       <c r="H5" s="2">
-        <v>1</v>
-      </c>
-      <c r="I5" s="2"/>
+        <v>0</v>
+      </c>
+      <c r="I5" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:9" ht="15">
       <c r="A6" s="2" t="s">
@@ -888,13 +942,23 @@
       <c r="C6" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
+      <c r="D6" s="2">
+        <v>0</v>
+      </c>
+      <c r="E6" s="2">
+        <v>1</v>
+      </c>
+      <c r="F6" s="2">
+        <v>1</v>
+      </c>
+      <c r="G6" s="2">
+        <v>1</v>
+      </c>
+      <c r="H6" s="2">
+        <v>1</v>
+      </c>
       <c r="I6" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15">
@@ -904,13 +968,27 @@
       <c r="B7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
+      <c r="C7" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D7" s="2">
+        <v>0</v>
+      </c>
+      <c r="E7" s="2">
+        <v>1</v>
+      </c>
+      <c r="F7" s="2">
+        <v>1</v>
+      </c>
+      <c r="G7" s="2">
+        <v>1</v>
+      </c>
+      <c r="H7" s="2">
+        <v>1</v>
+      </c>
+      <c r="I7" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:9" ht="15">
       <c r="A8" s="2" t="s">
@@ -919,13 +997,27 @@
       <c r="B8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
+      <c r="C8" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D8" s="2">
+        <v>0</v>
+      </c>
+      <c r="E8" s="2">
+        <v>1</v>
+      </c>
+      <c r="F8" s="2">
+        <v>1</v>
+      </c>
+      <c r="G8" s="2">
+        <v>1</v>
+      </c>
+      <c r="H8" s="2">
+        <v>1</v>
+      </c>
+      <c r="I8" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:9" ht="15">
       <c r="A9" s="2" t="s">
@@ -934,12 +1026,24 @@
       <c r="B9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
+      <c r="C9" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D9" s="2">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2">
+        <v>2</v>
+      </c>
+      <c r="F9" s="2">
+        <v>2</v>
+      </c>
+      <c r="G9" s="2">
+        <v>2</v>
+      </c>
+      <c r="H9" s="2">
+        <v>2</v>
+      </c>
       <c r="I9" s="2">
         <v>1</v>
       </c>
@@ -951,13 +1055,27 @@
       <c r="B10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
+      <c r="C10" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D10" s="2">
+        <v>0</v>
+      </c>
+      <c r="E10" s="2">
+        <v>1</v>
+      </c>
+      <c r="F10" s="2">
+        <v>1</v>
+      </c>
+      <c r="G10" s="2">
+        <v>1</v>
+      </c>
+      <c r="H10" s="2">
+        <v>1</v>
+      </c>
+      <c r="I10" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:9" ht="15">
       <c r="A11" s="2" t="s">
@@ -966,13 +1084,27 @@
       <c r="B11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
+      <c r="C11" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D11" s="2">
+        <v>1</v>
+      </c>
+      <c r="E11" s="2">
+        <v>1</v>
+      </c>
+      <c r="F11" s="2">
+        <v>1</v>
+      </c>
+      <c r="G11" s="2">
+        <v>1</v>
+      </c>
+      <c r="H11" s="2">
+        <v>1</v>
+      </c>
+      <c r="I11" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="12" spans="1:9" ht="15">
       <c r="A12" s="2" t="s">
@@ -981,13 +1113,27 @@
       <c r="B12" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
+      <c r="C12" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D12" s="2">
+        <v>0</v>
+      </c>
+      <c r="E12" s="2">
+        <v>1</v>
+      </c>
+      <c r="F12" s="2">
+        <v>1</v>
+      </c>
+      <c r="G12" s="2">
+        <v>1</v>
+      </c>
+      <c r="H12" s="2">
+        <v>1</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="1:9" ht="15">
       <c r="A13" s="2" t="s">
@@ -996,13 +1142,27 @@
       <c r="B13" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
+      <c r="C13" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D13" s="2">
+        <v>1</v>
+      </c>
+      <c r="E13" s="2">
+        <v>1</v>
+      </c>
+      <c r="F13" s="2">
+        <v>1</v>
+      </c>
+      <c r="G13" s="2">
+        <v>1</v>
+      </c>
+      <c r="H13" s="2">
+        <v>1</v>
+      </c>
+      <c r="I13" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="14" spans="1:9" ht="15">
       <c r="A14" s="2" t="s">
@@ -1011,13 +1171,27 @@
       <c r="B14" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
+      <c r="C14" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D14" s="2">
+        <v>0</v>
+      </c>
+      <c r="E14" s="2">
+        <v>2</v>
+      </c>
+      <c r="F14" s="2">
+        <v>2</v>
+      </c>
+      <c r="G14" s="2">
+        <v>1</v>
+      </c>
+      <c r="H14" s="2">
+        <v>1</v>
+      </c>
+      <c r="I14" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="15" spans="1:9" ht="15">
       <c r="A15" s="2" t="s">
@@ -1026,13 +1200,27 @@
       <c r="B15" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
+      <c r="C15" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D15" s="2">
+        <v>0</v>
+      </c>
+      <c r="E15" s="2">
+        <v>2</v>
+      </c>
+      <c r="F15" s="2">
+        <v>2</v>
+      </c>
+      <c r="G15" s="2">
+        <v>2</v>
+      </c>
+      <c r="H15" s="2">
+        <v>1</v>
+      </c>
+      <c r="I15" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="16" spans="1:9" ht="15">
       <c r="A16" s="2" t="s">
@@ -1041,13 +1229,27 @@
       <c r="B16" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
+      <c r="C16" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D16" s="2">
+        <v>0</v>
+      </c>
+      <c r="E16" s="2">
+        <v>2</v>
+      </c>
+      <c r="F16" s="2">
+        <v>2</v>
+      </c>
+      <c r="G16" s="2">
+        <v>1</v>
+      </c>
+      <c r="H16" s="2">
+        <v>1</v>
+      </c>
+      <c r="I16" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="17" spans="1:9" ht="15">
       <c r="A17" s="2" t="s">
@@ -1056,13 +1258,27 @@
       <c r="B17" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
+      <c r="C17" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D17" s="2">
+        <v>2</v>
+      </c>
+      <c r="E17" s="2">
+        <v>2</v>
+      </c>
+      <c r="F17" s="2">
+        <v>2</v>
+      </c>
+      <c r="G17" s="2">
+        <v>2</v>
+      </c>
+      <c r="H17" s="2">
+        <v>2</v>
+      </c>
+      <c r="I17" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="18" spans="1:9" ht="15">
       <c r="A18" s="2" t="s">
@@ -1071,13 +1287,27 @@
       <c r="B18" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
+      <c r="C18" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D18" s="2">
+        <v>0</v>
+      </c>
+      <c r="E18" s="2">
+        <v>1</v>
+      </c>
+      <c r="F18" s="2">
+        <v>2</v>
+      </c>
+      <c r="G18" s="2">
+        <v>2</v>
+      </c>
+      <c r="H18" s="2">
+        <v>1</v>
+      </c>
+      <c r="I18" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="19" spans="1:9" ht="15">
       <c r="A19" s="2" t="s">
@@ -1086,13 +1316,27 @@
       <c r="B19" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
+      <c r="C19" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D19" s="2">
+        <v>1</v>
+      </c>
+      <c r="E19" s="2">
+        <v>1</v>
+      </c>
+      <c r="F19" s="2">
+        <v>1</v>
+      </c>
+      <c r="G19" s="2">
+        <v>1</v>
+      </c>
+      <c r="H19" s="2">
+        <v>1</v>
+      </c>
+      <c r="I19" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="20" spans="1:9" ht="15">
       <c r="A20" s="2" t="s">
@@ -1101,13 +1345,27 @@
       <c r="B20" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
+      <c r="C20" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D20" s="2">
+        <v>0</v>
+      </c>
+      <c r="E20" s="2">
+        <v>2</v>
+      </c>
+      <c r="F20" s="2">
+        <v>2</v>
+      </c>
+      <c r="G20" s="2">
+        <v>1</v>
+      </c>
+      <c r="H20" s="2">
+        <v>2</v>
+      </c>
+      <c r="I20" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="21" spans="1:9" ht="15">
       <c r="A21" s="2" t="s">
@@ -1116,13 +1374,27 @@
       <c r="B21" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
+      <c r="C21" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D21" s="2">
+        <v>1</v>
+      </c>
+      <c r="E21" s="2">
+        <v>0</v>
+      </c>
+      <c r="F21" s="2">
+        <v>1</v>
+      </c>
+      <c r="G21" s="2">
+        <v>2</v>
+      </c>
+      <c r="H21" s="2">
+        <v>2</v>
+      </c>
+      <c r="I21" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="22" spans="1:9" ht="15">
       <c r="A22" s="2" t="s">
@@ -1131,13 +1403,27 @@
       <c r="B22" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
+      <c r="C22" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D22" s="2">
+        <v>1</v>
+      </c>
+      <c r="E22" s="2">
+        <v>2</v>
+      </c>
+      <c r="F22" s="2">
+        <v>1</v>
+      </c>
+      <c r="G22" s="2">
+        <v>2</v>
+      </c>
+      <c r="H22" s="2">
+        <v>0</v>
+      </c>
+      <c r="I22" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="23" spans="1:9" ht="15">
       <c r="A23" s="2" t="s">
@@ -1146,13 +1432,27 @@
       <c r="B23" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
+      <c r="C23" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D23" s="2">
+        <v>0</v>
+      </c>
+      <c r="E23" s="2">
+        <v>2</v>
+      </c>
+      <c r="F23" s="2">
+        <v>2</v>
+      </c>
+      <c r="G23" s="2">
+        <v>2</v>
+      </c>
+      <c r="H23" s="2">
+        <v>1</v>
+      </c>
+      <c r="I23" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="24" spans="1:9" ht="15">
       <c r="A24" s="2" t="s">
@@ -1161,13 +1461,27 @@
       <c r="B24" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
+      <c r="C24" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D24" s="2">
+        <v>0</v>
+      </c>
+      <c r="E24" s="2">
+        <v>1</v>
+      </c>
+      <c r="F24" s="2">
+        <v>1</v>
+      </c>
+      <c r="G24" s="2">
+        <v>2</v>
+      </c>
+      <c r="H24" s="2">
+        <v>1</v>
+      </c>
+      <c r="I24" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="25" spans="1:9" ht="15">
       <c r="A25" s="2" t="s">
@@ -1176,13 +1490,27 @@
       <c r="B25" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
+      <c r="C25" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D25" s="2">
+        <v>0</v>
+      </c>
+      <c r="E25" s="2">
+        <v>1</v>
+      </c>
+      <c r="F25" s="2">
+        <v>1</v>
+      </c>
+      <c r="G25" s="2">
+        <v>2</v>
+      </c>
+      <c r="H25" s="2">
+        <v>0</v>
+      </c>
+      <c r="I25" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="26" spans="1:9" ht="15">
       <c r="A26" s="2" t="s">
@@ -1191,13 +1519,27 @@
       <c r="B26" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
+      <c r="C26" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D26" s="2">
+        <v>1</v>
+      </c>
+      <c r="E26" s="2">
+        <v>1</v>
+      </c>
+      <c r="F26" s="2">
+        <v>1</v>
+      </c>
+      <c r="G26" s="2">
+        <v>2</v>
+      </c>
+      <c r="H26" s="2">
+        <v>0</v>
+      </c>
+      <c r="I26" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="27" spans="1:9" ht="15">
       <c r="A27" s="2" t="s">
@@ -1206,13 +1548,27 @@
       <c r="B27" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
+      <c r="C27" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D27" s="2">
+        <v>0</v>
+      </c>
+      <c r="E27" s="2">
+        <v>0</v>
+      </c>
+      <c r="F27" s="2">
+        <v>0</v>
+      </c>
+      <c r="G27" s="2">
+        <v>2</v>
+      </c>
+      <c r="H27" s="2">
+        <v>0</v>
+      </c>
+      <c r="I27" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="28" spans="1:9" ht="15">
       <c r="A28" s="2" t="s">
@@ -1221,13 +1577,27 @@
       <c r="B28" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
+      <c r="C28" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D28" s="2">
+        <v>0</v>
+      </c>
+      <c r="E28" s="2">
+        <v>0</v>
+      </c>
+      <c r="F28" s="2">
+        <v>0</v>
+      </c>
+      <c r="G28" s="2">
+        <v>2</v>
+      </c>
+      <c r="H28" s="2">
+        <v>0</v>
+      </c>
+      <c r="I28" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="29" spans="1:9" ht="15">
       <c r="A29" s="2" t="s">
@@ -1236,13 +1606,27 @@
       <c r="B29" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
+      <c r="C29" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D29" s="2">
+        <v>0</v>
+      </c>
+      <c r="E29" s="2">
+        <v>0</v>
+      </c>
+      <c r="F29" s="2">
+        <v>0</v>
+      </c>
+      <c r="G29" s="2">
+        <v>2</v>
+      </c>
+      <c r="H29" s="2">
+        <v>0</v>
+      </c>
+      <c r="I29" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="30" spans="1:9" ht="15">
       <c r="A30" s="2" t="s">
@@ -1251,13 +1635,27 @@
       <c r="B30" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
+      <c r="C30" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D30" s="2">
+        <v>0</v>
+      </c>
+      <c r="E30" s="2">
+        <v>1</v>
+      </c>
+      <c r="F30" s="2">
+        <v>1</v>
+      </c>
+      <c r="G30" s="2">
+        <v>2</v>
+      </c>
+      <c r="H30" s="2">
+        <v>1</v>
+      </c>
+      <c r="I30" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="31" spans="1:9" ht="15">
       <c r="A31" s="2" t="s">
@@ -1266,13 +1664,27 @@
       <c r="B31" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="2"/>
-      <c r="I31" s="2"/>
+      <c r="C31" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D31" s="2">
+        <v>2</v>
+      </c>
+      <c r="E31" s="2">
+        <v>1</v>
+      </c>
+      <c r="F31" s="2">
+        <v>1</v>
+      </c>
+      <c r="G31" s="2">
+        <v>2</v>
+      </c>
+      <c r="H31" s="2">
+        <v>2</v>
+      </c>
+      <c r="I31" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="32" spans="1:9" ht="15">
       <c r="A32" s="2" t="s">
@@ -1281,13 +1693,27 @@
       <c r="B32" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
-      <c r="H32" s="2"/>
-      <c r="I32" s="2"/>
+      <c r="C32" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D32" s="2">
+        <v>2</v>
+      </c>
+      <c r="E32" s="2">
+        <v>2</v>
+      </c>
+      <c r="F32" s="2">
+        <v>2</v>
+      </c>
+      <c r="G32" s="2">
+        <v>2</v>
+      </c>
+      <c r="H32" s="2">
+        <v>1</v>
+      </c>
+      <c r="I32" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="33" spans="1:9" ht="15">
       <c r="A33" s="2" t="s">
@@ -1296,13 +1722,27 @@
       <c r="B33" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
+      <c r="C33" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D33" s="2">
+        <v>1</v>
+      </c>
+      <c r="E33" s="2">
+        <v>1</v>
+      </c>
+      <c r="F33" s="2">
+        <v>1</v>
+      </c>
+      <c r="G33" s="2">
+        <v>1</v>
+      </c>
+      <c r="H33" s="2">
+        <v>1</v>
+      </c>
+      <c r="I33" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="34" spans="1:9" ht="15">
       <c r="A34" s="2" t="s">
@@ -1311,13 +1751,27 @@
       <c r="B34" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-      <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
+      <c r="C34" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D34" s="2">
+        <v>2</v>
+      </c>
+      <c r="E34" s="2">
+        <v>1</v>
+      </c>
+      <c r="F34" s="2">
+        <v>1</v>
+      </c>
+      <c r="G34" s="2">
+        <v>1</v>
+      </c>
+      <c r="H34" s="2">
+        <v>1</v>
+      </c>
+      <c r="I34" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="35" spans="1:9" ht="15">
       <c r="A35" s="2" t="s">
@@ -1326,13 +1780,27 @@
       <c r="B35" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-      <c r="H35" s="2"/>
-      <c r="I35" s="2"/>
+      <c r="C35" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D35" s="2">
+        <v>1</v>
+      </c>
+      <c r="E35" s="2">
+        <v>1</v>
+      </c>
+      <c r="F35" s="2">
+        <v>1</v>
+      </c>
+      <c r="G35" s="2">
+        <v>1</v>
+      </c>
+      <c r="H35" s="2">
+        <v>1</v>
+      </c>
+      <c r="I35" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="36" spans="1:9" ht="15">
       <c r="A36" s="2" t="s">
@@ -1341,13 +1809,27 @@
       <c r="B36" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-      <c r="H36" s="2"/>
-      <c r="I36" s="2"/>
+      <c r="C36" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D36" s="2">
+        <v>1</v>
+      </c>
+      <c r="E36" s="2">
+        <v>1</v>
+      </c>
+      <c r="F36" s="2">
+        <v>1</v>
+      </c>
+      <c r="G36" s="2">
+        <v>1</v>
+      </c>
+      <c r="H36" s="2">
+        <v>1</v>
+      </c>
+      <c r="I36" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="37" spans="1:9" ht="15">
       <c r="A37" s="2" t="s">
@@ -1356,13 +1838,27 @@
       <c r="B37" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
-      <c r="H37" s="2"/>
-      <c r="I37" s="2"/>
+      <c r="C37" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D37" s="2">
+        <v>2</v>
+      </c>
+      <c r="E37" s="2">
+        <v>1</v>
+      </c>
+      <c r="F37" s="2">
+        <v>1</v>
+      </c>
+      <c r="G37" s="2">
+        <v>2</v>
+      </c>
+      <c r="H37" s="2">
+        <v>1</v>
+      </c>
+      <c r="I37" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="38" spans="1:9" ht="15">
       <c r="A38" s="2" t="s">
@@ -1371,13 +1867,27 @@
       <c r="B38" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="2"/>
-      <c r="H38" s="2"/>
-      <c r="I38" s="2"/>
+      <c r="C38" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D38" s="2">
+        <v>2</v>
+      </c>
+      <c r="E38" s="2">
+        <v>2</v>
+      </c>
+      <c r="F38" s="2">
+        <v>2</v>
+      </c>
+      <c r="G38" s="2">
+        <v>2</v>
+      </c>
+      <c r="H38" s="2">
+        <v>2</v>
+      </c>
+      <c r="I38" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="39" spans="1:9" ht="15">
       <c r="A39" s="2" t="s">
@@ -1386,13 +1896,27 @@
       <c r="B39" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
-      <c r="G39" s="2"/>
-      <c r="H39" s="2"/>
-      <c r="I39" s="2"/>
+      <c r="C39" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D39" s="2">
+        <v>1</v>
+      </c>
+      <c r="E39" s="2">
+        <v>2</v>
+      </c>
+      <c r="F39" s="2">
+        <v>2</v>
+      </c>
+      <c r="G39" s="2">
+        <v>2</v>
+      </c>
+      <c r="H39" s="2">
+        <v>1</v>
+      </c>
+      <c r="I39" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="40" spans="1:9" ht="15">
       <c r="A40" s="2" t="s">
@@ -1401,13 +1925,27 @@
       <c r="B40" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
-      <c r="F40" s="2"/>
-      <c r="G40" s="2"/>
-      <c r="H40" s="2"/>
-      <c r="I40" s="2"/>
+      <c r="C40" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D40" s="2">
+        <v>2</v>
+      </c>
+      <c r="E40" s="2">
+        <v>2</v>
+      </c>
+      <c r="F40" s="2">
+        <v>2</v>
+      </c>
+      <c r="G40" s="2">
+        <v>2</v>
+      </c>
+      <c r="H40" s="2">
+        <v>1</v>
+      </c>
+      <c r="I40" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="41" spans="1:9" ht="15">
       <c r="A41" s="2" t="s">
@@ -1416,13 +1954,27 @@
       <c r="B41" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
-      <c r="F41" s="2"/>
-      <c r="G41" s="2"/>
-      <c r="H41" s="2"/>
-      <c r="I41" s="2"/>
+      <c r="C41" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D41" s="2">
+        <v>1</v>
+      </c>
+      <c r="E41" s="2">
+        <v>2</v>
+      </c>
+      <c r="F41" s="2">
+        <v>2</v>
+      </c>
+      <c r="G41" s="2">
+        <v>1</v>
+      </c>
+      <c r="H41" s="2">
+        <v>1</v>
+      </c>
+      <c r="I41" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="42" spans="1:9" ht="15">
       <c r="A42" s="2" t="s">
@@ -1431,13 +1983,27 @@
       <c r="B42" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
-      <c r="E42" s="2"/>
-      <c r="F42" s="2"/>
-      <c r="G42" s="2"/>
-      <c r="H42" s="2"/>
-      <c r="I42" s="2"/>
+      <c r="C42" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D42" s="2">
+        <v>2</v>
+      </c>
+      <c r="E42" s="2">
+        <v>1</v>
+      </c>
+      <c r="F42" s="2">
+        <v>1</v>
+      </c>
+      <c r="G42" s="2">
+        <v>1</v>
+      </c>
+      <c r="H42" s="2">
+        <v>2</v>
+      </c>
+      <c r="I42" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="43" spans="1:9" ht="15">
       <c r="A43" s="2" t="s">
@@ -1446,13 +2012,27 @@
       <c r="B43" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-      <c r="E43" s="2"/>
-      <c r="F43" s="2"/>
-      <c r="G43" s="2"/>
-      <c r="H43" s="2"/>
-      <c r="I43" s="2"/>
+      <c r="C43" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D43" s="2">
+        <v>2</v>
+      </c>
+      <c r="E43" s="2">
+        <v>1</v>
+      </c>
+      <c r="F43" s="2">
+        <v>1</v>
+      </c>
+      <c r="G43" s="2">
+        <v>2</v>
+      </c>
+      <c r="H43" s="2">
+        <v>2</v>
+      </c>
+      <c r="I43" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="44" spans="1:9" ht="15">
       <c r="A44" s="2" t="s">
@@ -1461,13 +2041,27 @@
       <c r="B44" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
-      <c r="F44" s="2"/>
-      <c r="G44" s="2"/>
-      <c r="H44" s="2"/>
-      <c r="I44" s="2"/>
+      <c r="C44" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D44" s="2">
+        <v>2</v>
+      </c>
+      <c r="E44" s="2">
+        <v>1</v>
+      </c>
+      <c r="F44" s="2">
+        <v>1</v>
+      </c>
+      <c r="G44" s="2">
+        <v>2</v>
+      </c>
+      <c r="H44" s="2">
+        <v>2</v>
+      </c>
+      <c r="I44" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="45" spans="1:9" ht="15">
       <c r="A45" s="2" t="s">
@@ -1476,13 +2070,27 @@
       <c r="B45" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-      <c r="F45" s="2"/>
-      <c r="G45" s="2"/>
-      <c r="H45" s="2"/>
-      <c r="I45" s="2"/>
+      <c r="C45" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D45" s="2">
+        <v>2</v>
+      </c>
+      <c r="E45" s="2">
+        <v>1</v>
+      </c>
+      <c r="F45" s="2">
+        <v>1</v>
+      </c>
+      <c r="G45" s="2">
+        <v>2</v>
+      </c>
+      <c r="H45" s="2">
+        <v>2</v>
+      </c>
+      <c r="I45" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="46" spans="1:9" ht="15">
       <c r="A46" s="2" t="s">
@@ -1491,13 +2099,27 @@
       <c r="B46" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
-      <c r="E46" s="2"/>
-      <c r="F46" s="2"/>
-      <c r="G46" s="2"/>
-      <c r="H46" s="2"/>
-      <c r="I46" s="2"/>
+      <c r="C46" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D46" s="2">
+        <v>1</v>
+      </c>
+      <c r="E46" s="2">
+        <v>1</v>
+      </c>
+      <c r="F46" s="2">
+        <v>1</v>
+      </c>
+      <c r="G46" s="2">
+        <v>1</v>
+      </c>
+      <c r="H46" s="2">
+        <v>1</v>
+      </c>
+      <c r="I46" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="47" spans="1:9" ht="15">
       <c r="A47" s="2" t="s">
@@ -1506,13 +2128,27 @@
       <c r="B47" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
-      <c r="F47" s="2"/>
-      <c r="G47" s="2"/>
-      <c r="H47" s="2"/>
-      <c r="I47" s="2"/>
+      <c r="C47" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D47" s="2">
+        <v>2</v>
+      </c>
+      <c r="E47" s="2">
+        <v>1</v>
+      </c>
+      <c r="F47" s="2">
+        <v>1</v>
+      </c>
+      <c r="G47" s="2">
+        <v>1</v>
+      </c>
+      <c r="H47" s="2">
+        <v>1</v>
+      </c>
+      <c r="I47" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="48" spans="1:9" ht="15">
       <c r="A48" s="2" t="s">
@@ -1521,13 +2157,27 @@
       <c r="B48" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2"/>
-      <c r="E48" s="2"/>
-      <c r="F48" s="2"/>
-      <c r="G48" s="2"/>
-      <c r="H48" s="2"/>
-      <c r="I48" s="2"/>
+      <c r="C48" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D48" s="2">
+        <v>2</v>
+      </c>
+      <c r="E48" s="2">
+        <v>0</v>
+      </c>
+      <c r="F48" s="2">
+        <v>0</v>
+      </c>
+      <c r="G48" s="2">
+        <v>0</v>
+      </c>
+      <c r="H48" s="2">
+        <v>2</v>
+      </c>
+      <c r="I48" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="49" spans="1:9" ht="15">
       <c r="A49" s="2" t="s">
@@ -1536,13 +2186,27 @@
       <c r="B49" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
-      <c r="E49" s="2"/>
-      <c r="F49" s="2"/>
-      <c r="G49" s="2"/>
-      <c r="H49" s="2"/>
-      <c r="I49" s="2"/>
+      <c r="C49" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D49" s="2">
+        <v>1</v>
+      </c>
+      <c r="E49" s="2">
+        <v>1</v>
+      </c>
+      <c r="F49" s="2">
+        <v>1</v>
+      </c>
+      <c r="G49" s="2">
+        <v>1</v>
+      </c>
+      <c r="H49" s="2">
+        <v>1</v>
+      </c>
+      <c r="I49" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="50" spans="1:9" ht="15">
       <c r="A50" s="2" t="s">
@@ -1551,13 +2215,27 @@
       <c r="B50" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C50" s="2"/>
-      <c r="D50" s="2"/>
-      <c r="E50" s="2"/>
-      <c r="F50" s="2"/>
-      <c r="G50" s="2"/>
-      <c r="H50" s="2"/>
-      <c r="I50" s="2"/>
+      <c r="C50" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D50" s="2">
+        <v>0</v>
+      </c>
+      <c r="E50" s="2">
+        <v>0</v>
+      </c>
+      <c r="F50" s="2">
+        <v>2</v>
+      </c>
+      <c r="G50" s="2">
+        <v>0</v>
+      </c>
+      <c r="H50" s="2">
+        <v>0</v>
+      </c>
+      <c r="I50" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="51" spans="1:9" ht="15">
       <c r="A51" s="2" t="s">
@@ -1566,13 +2244,27 @@
       <c r="B51" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-      <c r="E51" s="2"/>
-      <c r="F51" s="2"/>
-      <c r="G51" s="2"/>
-      <c r="H51" s="2"/>
-      <c r="I51" s="2"/>
+      <c r="C51" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D51" s="2">
+        <v>0</v>
+      </c>
+      <c r="E51" s="2">
+        <v>0</v>
+      </c>
+      <c r="F51" s="2">
+        <v>2</v>
+      </c>
+      <c r="G51" s="2">
+        <v>0</v>
+      </c>
+      <c r="H51" s="2">
+        <v>0</v>
+      </c>
+      <c r="I51" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="52" spans="1:9" ht="15">
       <c r="A52" s="2" t="s">
@@ -1581,13 +2273,27 @@
       <c r="B52" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C52" s="2"/>
-      <c r="D52" s="2"/>
-      <c r="E52" s="2"/>
-      <c r="F52" s="2"/>
-      <c r="G52" s="2"/>
-      <c r="H52" s="2"/>
-      <c r="I52" s="2"/>
+      <c r="C52" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D52" s="2">
+        <v>0</v>
+      </c>
+      <c r="E52" s="2">
+        <v>0</v>
+      </c>
+      <c r="F52" s="2">
+        <v>2</v>
+      </c>
+      <c r="G52" s="2">
+        <v>0</v>
+      </c>
+      <c r="H52" s="2">
+        <v>0</v>
+      </c>
+      <c r="I52" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="53" spans="1:9" ht="15">
       <c r="A53" s="2" t="s">
@@ -1596,13 +2302,27 @@
       <c r="B53" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C53" s="2"/>
-      <c r="D53" s="2"/>
-      <c r="E53" s="2"/>
-      <c r="F53" s="2"/>
-      <c r="G53" s="2"/>
-      <c r="H53" s="2"/>
-      <c r="I53" s="2"/>
+      <c r="C53" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D53" s="2">
+        <v>0</v>
+      </c>
+      <c r="E53" s="2">
+        <v>0</v>
+      </c>
+      <c r="F53" s="2">
+        <v>2</v>
+      </c>
+      <c r="G53" s="2">
+        <v>0</v>
+      </c>
+      <c r="H53" s="2">
+        <v>0</v>
+      </c>
+      <c r="I53" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="54" spans="1:9" ht="15">
       <c r="A54" s="2" t="s">
@@ -1611,13 +2331,27 @@
       <c r="B54" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C54" s="2"/>
-      <c r="D54" s="2"/>
-      <c r="E54" s="2"/>
-      <c r="F54" s="2"/>
-      <c r="G54" s="2"/>
-      <c r="H54" s="2"/>
-      <c r="I54" s="2"/>
+      <c r="C54" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D54" s="2">
+        <v>1</v>
+      </c>
+      <c r="E54" s="2">
+        <v>1</v>
+      </c>
+      <c r="F54" s="2">
+        <v>1</v>
+      </c>
+      <c r="G54" s="2">
+        <v>1</v>
+      </c>
+      <c r="H54" s="2">
+        <v>1</v>
+      </c>
+      <c r="I54" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="55" spans="1:9" ht="15">
       <c r="A55" s="2" t="s">
@@ -1626,13 +2360,27 @@
       <c r="B55" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C55" s="2"/>
-      <c r="D55" s="2"/>
-      <c r="E55" s="2"/>
-      <c r="F55" s="2"/>
-      <c r="G55" s="2"/>
-      <c r="H55" s="2"/>
-      <c r="I55" s="2"/>
+      <c r="C55" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D55" s="2">
+        <v>1</v>
+      </c>
+      <c r="E55" s="2">
+        <v>1</v>
+      </c>
+      <c r="F55" s="2">
+        <v>1</v>
+      </c>
+      <c r="G55" s="2">
+        <v>1</v>
+      </c>
+      <c r="H55" s="2">
+        <v>1</v>
+      </c>
+      <c r="I55" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="56" spans="1:9" ht="15">
       <c r="A56" s="2" t="s">
@@ -1641,13 +2389,27 @@
       <c r="B56" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C56" s="2"/>
-      <c r="D56" s="2"/>
-      <c r="E56" s="2"/>
-      <c r="F56" s="2"/>
-      <c r="G56" s="2"/>
-      <c r="H56" s="2"/>
-      <c r="I56" s="2"/>
+      <c r="C56" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D56" s="2">
+        <v>1</v>
+      </c>
+      <c r="E56" s="2">
+        <v>1</v>
+      </c>
+      <c r="F56" s="2">
+        <v>1</v>
+      </c>
+      <c r="G56" s="2">
+        <v>1</v>
+      </c>
+      <c r="H56" s="2">
+        <v>1</v>
+      </c>
+      <c r="I56" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="57" spans="1:9" ht="15">
       <c r="A57" s="2" t="s">
@@ -1656,13 +2418,27 @@
       <c r="B57" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C57" s="2"/>
-      <c r="D57" s="2"/>
-      <c r="E57" s="2"/>
-      <c r="F57" s="2"/>
-      <c r="G57" s="2"/>
-      <c r="H57" s="2"/>
-      <c r="I57" s="2"/>
+      <c r="C57" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D57" s="2">
+        <v>2</v>
+      </c>
+      <c r="E57" s="2">
+        <v>1</v>
+      </c>
+      <c r="F57" s="2">
+        <v>1</v>
+      </c>
+      <c r="G57" s="2">
+        <v>1</v>
+      </c>
+      <c r="H57" s="2">
+        <v>2</v>
+      </c>
+      <c r="I57" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="58" spans="1:9" ht="15">
       <c r="A58" s="2" t="s">
@@ -1671,13 +2447,27 @@
       <c r="B58" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C58" s="2"/>
-      <c r="D58" s="2"/>
-      <c r="E58" s="2"/>
-      <c r="F58" s="2"/>
-      <c r="G58" s="2"/>
-      <c r="H58" s="2"/>
-      <c r="I58" s="2"/>
+      <c r="C58" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D58" s="2">
+        <v>1</v>
+      </c>
+      <c r="E58" s="2">
+        <v>1</v>
+      </c>
+      <c r="F58" s="2">
+        <v>1</v>
+      </c>
+      <c r="G58" s="2">
+        <v>1</v>
+      </c>
+      <c r="H58" s="2">
+        <v>1</v>
+      </c>
+      <c r="I58" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="59" spans="1:9" ht="15">
       <c r="A59" s="2" t="s">
@@ -1686,13 +2476,27 @@
       <c r="B59" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C59" s="2"/>
-      <c r="D59" s="2"/>
-      <c r="E59" s="2"/>
-      <c r="F59" s="2"/>
-      <c r="G59" s="2"/>
-      <c r="H59" s="2"/>
-      <c r="I59" s="2"/>
+      <c r="C59" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D59" s="2">
+        <v>1</v>
+      </c>
+      <c r="E59" s="2">
+        <v>1</v>
+      </c>
+      <c r="F59" s="2">
+        <v>1</v>
+      </c>
+      <c r="G59" s="2">
+        <v>1</v>
+      </c>
+      <c r="H59" s="2">
+        <v>1</v>
+      </c>
+      <c r="I59" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="60" spans="1:9" ht="15">
       <c r="A60" s="2" t="s">
@@ -1701,13 +2505,27 @@
       <c r="B60" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C60" s="2"/>
-      <c r="D60" s="2"/>
-      <c r="E60" s="2"/>
-      <c r="F60" s="2"/>
-      <c r="G60" s="2"/>
-      <c r="H60" s="2"/>
-      <c r="I60" s="2"/>
+      <c r="C60" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D60" s="2">
+        <v>0</v>
+      </c>
+      <c r="E60" s="2">
+        <v>1</v>
+      </c>
+      <c r="F60" s="2">
+        <v>1</v>
+      </c>
+      <c r="G60" s="2">
+        <v>2</v>
+      </c>
+      <c r="H60" s="2">
+        <v>0</v>
+      </c>
+      <c r="I60" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="61" spans="1:9" ht="15">
       <c r="A61" s="2" t="s">
@@ -1716,13 +2534,27 @@
       <c r="B61" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C61" s="2"/>
-      <c r="D61" s="2"/>
-      <c r="E61" s="2"/>
-      <c r="F61" s="2"/>
-      <c r="G61" s="2"/>
-      <c r="H61" s="2"/>
-      <c r="I61" s="2"/>
+      <c r="C61" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D61" s="2">
+        <v>1</v>
+      </c>
+      <c r="E61" s="2">
+        <v>1</v>
+      </c>
+      <c r="F61" s="2">
+        <v>1</v>
+      </c>
+      <c r="G61" s="2">
+        <v>1</v>
+      </c>
+      <c r="H61" s="2">
+        <v>1</v>
+      </c>
+      <c r="I61" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="62" spans="1:9" ht="15">
       <c r="A62" s="2" t="s">
@@ -1731,13 +2563,27 @@
       <c r="B62" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C62" s="2"/>
-      <c r="D62" s="2"/>
-      <c r="E62" s="2"/>
-      <c r="F62" s="2"/>
-      <c r="G62" s="2"/>
-      <c r="H62" s="2"/>
-      <c r="I62" s="2"/>
+      <c r="C62" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D62" s="2">
+        <v>1</v>
+      </c>
+      <c r="E62" s="2">
+        <v>2</v>
+      </c>
+      <c r="F62" s="2">
+        <v>2</v>
+      </c>
+      <c r="G62" s="2">
+        <v>2</v>
+      </c>
+      <c r="H62" s="2">
+        <v>0</v>
+      </c>
+      <c r="I62" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="63" spans="1:9" ht="15">
       <c r="A63" s="2" t="s">
@@ -1746,13 +2592,27 @@
       <c r="B63" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C63" s="2"/>
-      <c r="D63" s="2"/>
-      <c r="E63" s="2"/>
-      <c r="F63" s="2"/>
-      <c r="G63" s="2"/>
-      <c r="H63" s="2"/>
-      <c r="I63" s="2"/>
+      <c r="C63" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D63" s="2">
+        <v>2</v>
+      </c>
+      <c r="E63" s="2">
+        <v>1</v>
+      </c>
+      <c r="F63" s="2">
+        <v>2</v>
+      </c>
+      <c r="G63" s="2">
+        <v>2</v>
+      </c>
+      <c r="H63" s="2">
+        <v>2</v>
+      </c>
+      <c r="I63" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="64" spans="1:9" ht="15">
       <c r="A64" s="2" t="s">
@@ -1761,13 +2621,27 @@
       <c r="B64" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C64" s="2"/>
-      <c r="D64" s="2"/>
-      <c r="E64" s="2"/>
-      <c r="F64" s="2"/>
-      <c r="G64" s="2"/>
-      <c r="H64" s="2"/>
-      <c r="I64" s="2"/>
+      <c r="C64" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D64" s="2">
+        <v>1</v>
+      </c>
+      <c r="E64" s="2">
+        <v>2</v>
+      </c>
+      <c r="F64" s="2">
+        <v>2</v>
+      </c>
+      <c r="G64" s="2">
+        <v>1</v>
+      </c>
+      <c r="H64" s="2">
+        <v>0</v>
+      </c>
+      <c r="I64" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="65" spans="1:9" ht="15">
       <c r="A65" s="2" t="s">
@@ -1776,13 +2650,27 @@
       <c r="B65" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C65" s="2"/>
-      <c r="D65" s="2"/>
-      <c r="E65" s="2"/>
-      <c r="F65" s="2"/>
-      <c r="G65" s="2"/>
-      <c r="H65" s="2"/>
-      <c r="I65" s="2"/>
+      <c r="C65" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D65" s="2">
+        <v>1</v>
+      </c>
+      <c r="E65" s="2">
+        <v>2</v>
+      </c>
+      <c r="F65" s="2">
+        <v>2</v>
+      </c>
+      <c r="G65" s="2">
+        <v>1</v>
+      </c>
+      <c r="H65" s="2">
+        <v>0</v>
+      </c>
+      <c r="I65" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="66" spans="1:9" ht="15">
       <c r="A66" s="2" t="s">
@@ -1791,13 +2679,27 @@
       <c r="B66" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C66" s="2"/>
-      <c r="D66" s="2"/>
-      <c r="E66" s="2"/>
-      <c r="F66" s="2"/>
-      <c r="G66" s="2"/>
-      <c r="H66" s="2"/>
-      <c r="I66" s="2"/>
+      <c r="C66" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D66" s="2">
+        <v>1</v>
+      </c>
+      <c r="E66" s="2">
+        <v>2</v>
+      </c>
+      <c r="F66" s="2">
+        <v>2</v>
+      </c>
+      <c r="G66" s="2">
+        <v>2</v>
+      </c>
+      <c r="H66" s="2">
+        <v>1</v>
+      </c>
+      <c r="I66" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="67" spans="1:9" ht="15">
       <c r="A67" s="2" t="s">
@@ -1806,13 +2708,27 @@
       <c r="B67" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C67" s="2"/>
-      <c r="D67" s="2"/>
-      <c r="E67" s="2"/>
-      <c r="F67" s="2"/>
-      <c r="G67" s="2"/>
-      <c r="H67" s="2"/>
-      <c r="I67" s="2"/>
+      <c r="C67" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D67" s="2">
+        <v>0</v>
+      </c>
+      <c r="E67" s="2">
+        <v>2</v>
+      </c>
+      <c r="F67" s="2">
+        <v>2</v>
+      </c>
+      <c r="G67" s="2">
+        <v>1</v>
+      </c>
+      <c r="H67" s="2">
+        <v>0</v>
+      </c>
+      <c r="I67" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="68" spans="1:9" ht="15">
       <c r="A68" s="2" t="s">
@@ -1821,13 +2737,27 @@
       <c r="B68" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C68" s="2"/>
-      <c r="D68" s="2"/>
-      <c r="E68" s="2"/>
-      <c r="F68" s="2"/>
-      <c r="G68" s="2"/>
-      <c r="H68" s="2"/>
-      <c r="I68" s="2"/>
+      <c r="C68" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D68" s="2">
+        <v>1</v>
+      </c>
+      <c r="E68" s="2">
+        <v>1</v>
+      </c>
+      <c r="F68" s="2">
+        <v>1</v>
+      </c>
+      <c r="G68" s="2">
+        <v>1</v>
+      </c>
+      <c r="H68" s="2">
+        <v>1</v>
+      </c>
+      <c r="I68" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="69" spans="1:9" ht="15">
       <c r="A69" s="2" t="s">
@@ -1836,13 +2766,27 @@
       <c r="B69" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C69" s="2"/>
-      <c r="D69" s="2"/>
-      <c r="E69" s="2"/>
-      <c r="F69" s="2"/>
-      <c r="G69" s="2"/>
-      <c r="H69" s="2"/>
-      <c r="I69" s="2"/>
+      <c r="C69" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D69" s="2">
+        <v>2</v>
+      </c>
+      <c r="E69" s="2">
+        <v>1</v>
+      </c>
+      <c r="F69" s="2">
+        <v>1</v>
+      </c>
+      <c r="G69" s="2">
+        <v>1</v>
+      </c>
+      <c r="H69" s="2">
+        <v>2</v>
+      </c>
+      <c r="I69" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="70" spans="1:9" ht="15">
       <c r="A70" s="2" t="s">
@@ -1851,13 +2795,27 @@
       <c r="B70" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C70" s="2"/>
-      <c r="D70" s="2"/>
-      <c r="E70" s="2"/>
-      <c r="F70" s="2"/>
-      <c r="G70" s="2"/>
-      <c r="H70" s="2"/>
-      <c r="I70" s="2"/>
+      <c r="C70" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D70" s="2">
+        <v>1</v>
+      </c>
+      <c r="E70" s="2">
+        <v>2</v>
+      </c>
+      <c r="F70" s="2">
+        <v>2</v>
+      </c>
+      <c r="G70" s="2">
+        <v>2</v>
+      </c>
+      <c r="H70" s="2">
+        <v>1</v>
+      </c>
+      <c r="I70" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="71" spans="1:9" ht="15">
       <c r="A71" s="2" t="s">
@@ -1866,13 +2824,27 @@
       <c r="B71" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C71" s="2"/>
-      <c r="D71" s="2"/>
-      <c r="E71" s="2"/>
-      <c r="F71" s="2"/>
-      <c r="G71" s="2"/>
-      <c r="H71" s="2"/>
-      <c r="I71" s="2"/>
+      <c r="C71" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D71" s="2">
+        <v>1</v>
+      </c>
+      <c r="E71" s="2">
+        <v>1</v>
+      </c>
+      <c r="F71" s="2">
+        <v>2</v>
+      </c>
+      <c r="G71" s="2">
+        <v>2</v>
+      </c>
+      <c r="H71" s="2">
+        <v>1</v>
+      </c>
+      <c r="I71" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="72" spans="1:9" ht="15">
       <c r="A72" s="2" t="s">
@@ -1881,13 +2853,27 @@
       <c r="B72" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C72" s="2"/>
-      <c r="D72" s="2"/>
-      <c r="E72" s="2"/>
-      <c r="F72" s="2"/>
-      <c r="G72" s="2"/>
-      <c r="H72" s="2"/>
-      <c r="I72" s="2"/>
+      <c r="C72" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D72" s="2">
+        <v>1</v>
+      </c>
+      <c r="E72" s="2">
+        <v>2</v>
+      </c>
+      <c r="F72" s="2">
+        <v>2</v>
+      </c>
+      <c r="G72" s="2">
+        <v>2</v>
+      </c>
+      <c r="H72" s="2">
+        <v>1</v>
+      </c>
+      <c r="I72" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="73" spans="1:9" ht="15">
       <c r="A73" s="2" t="s">
@@ -1896,13 +2882,27 @@
       <c r="B73" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C73" s="2"/>
-      <c r="D73" s="2"/>
-      <c r="E73" s="2"/>
-      <c r="F73" s="2"/>
-      <c r="G73" s="2"/>
-      <c r="H73" s="2"/>
-      <c r="I73" s="2"/>
+      <c r="C73" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D73" s="2">
+        <v>1</v>
+      </c>
+      <c r="E73" s="2">
+        <v>1</v>
+      </c>
+      <c r="F73" s="2">
+        <v>2</v>
+      </c>
+      <c r="G73" s="2">
+        <v>2</v>
+      </c>
+      <c r="H73" s="2">
+        <v>1</v>
+      </c>
+      <c r="I73" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="74" spans="1:9" ht="15">
       <c r="A74" s="2" t="s">
@@ -1911,13 +2911,27 @@
       <c r="B74" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C74" s="2"/>
-      <c r="D74" s="2"/>
-      <c r="E74" s="2"/>
-      <c r="F74" s="2"/>
-      <c r="G74" s="2"/>
-      <c r="H74" s="2"/>
-      <c r="I74" s="2"/>
+      <c r="C74" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D74" s="2">
+        <v>2</v>
+      </c>
+      <c r="E74" s="2">
+        <v>1</v>
+      </c>
+      <c r="F74" s="2">
+        <v>2</v>
+      </c>
+      <c r="G74" s="2">
+        <v>2</v>
+      </c>
+      <c r="H74" s="2">
+        <v>1</v>
+      </c>
+      <c r="I74" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="75" spans="1:9" ht="15">
       <c r="A75" s="2" t="s">
@@ -1926,13 +2940,27 @@
       <c r="B75" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C75" s="2"/>
-      <c r="D75" s="2"/>
-      <c r="E75" s="2"/>
-      <c r="F75" s="2"/>
-      <c r="G75" s="2"/>
-      <c r="H75" s="2"/>
-      <c r="I75" s="2"/>
+      <c r="C75" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D75" s="2">
+        <v>2</v>
+      </c>
+      <c r="E75" s="2">
+        <v>1</v>
+      </c>
+      <c r="F75" s="2">
+        <v>1</v>
+      </c>
+      <c r="G75" s="2">
+        <v>2</v>
+      </c>
+      <c r="H75" s="2">
+        <v>1</v>
+      </c>
+      <c r="I75" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="76" spans="1:9" ht="15">
       <c r="A76" s="2" t="s">
@@ -1941,13 +2969,27 @@
       <c r="B76" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="C76" s="2"/>
-      <c r="D76" s="2"/>
-      <c r="E76" s="2"/>
-      <c r="F76" s="2"/>
-      <c r="G76" s="2"/>
-      <c r="H76" s="2"/>
-      <c r="I76" s="2"/>
+      <c r="C76" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D76" s="2">
+        <v>2</v>
+      </c>
+      <c r="E76" s="2">
+        <v>1</v>
+      </c>
+      <c r="F76" s="2">
+        <v>1</v>
+      </c>
+      <c r="G76" s="2">
+        <v>2</v>
+      </c>
+      <c r="H76" s="2">
+        <v>1</v>
+      </c>
+      <c r="I76" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="77" spans="1:9" ht="15">
       <c r="A77" s="2" t="s">
@@ -1956,13 +2998,27 @@
       <c r="B77" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C77" s="2"/>
-      <c r="D77" s="2"/>
-      <c r="E77" s="2"/>
-      <c r="F77" s="2"/>
-      <c r="G77" s="2"/>
-      <c r="H77" s="2"/>
-      <c r="I77" s="2"/>
+      <c r="C77" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D77" s="2">
+        <v>1</v>
+      </c>
+      <c r="E77" s="2">
+        <v>1</v>
+      </c>
+      <c r="F77" s="2">
+        <v>1</v>
+      </c>
+      <c r="G77" s="2">
+        <v>1</v>
+      </c>
+      <c r="H77" s="2">
+        <v>1</v>
+      </c>
+      <c r="I77" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="78" spans="1:9" ht="15">
       <c r="A78" s="2" t="s">
@@ -1971,13 +3027,27 @@
       <c r="B78" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C78" s="2"/>
-      <c r="D78" s="2"/>
-      <c r="E78" s="2"/>
-      <c r="F78" s="2"/>
-      <c r="G78" s="2"/>
-      <c r="H78" s="2"/>
-      <c r="I78" s="2"/>
+      <c r="C78" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D78" s="2">
+        <v>1</v>
+      </c>
+      <c r="E78" s="2">
+        <v>1</v>
+      </c>
+      <c r="F78" s="2">
+        <v>1</v>
+      </c>
+      <c r="G78" s="2">
+        <v>2</v>
+      </c>
+      <c r="H78" s="2">
+        <v>1</v>
+      </c>
+      <c r="I78" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="79" spans="1:9" ht="15">
       <c r="A79" s="2" t="s">
@@ -1986,13 +3056,27 @@
       <c r="B79" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C79" s="2"/>
-      <c r="D79" s="2"/>
-      <c r="E79" s="2"/>
-      <c r="F79" s="2"/>
-      <c r="G79" s="2"/>
-      <c r="H79" s="2"/>
-      <c r="I79" s="2"/>
+      <c r="C79" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D79" s="2">
+        <v>1</v>
+      </c>
+      <c r="E79" s="2">
+        <v>1</v>
+      </c>
+      <c r="F79" s="2">
+        <v>1</v>
+      </c>
+      <c r="G79" s="2">
+        <v>1</v>
+      </c>
+      <c r="H79" s="2">
+        <v>1</v>
+      </c>
+      <c r="I79" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="80" spans="1:9" ht="15">
       <c r="A80" s="2" t="s">
@@ -2001,13 +3085,27 @@
       <c r="B80" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C80" s="2"/>
-      <c r="D80" s="2"/>
-      <c r="E80" s="2"/>
-      <c r="F80" s="2"/>
-      <c r="G80" s="2"/>
-      <c r="H80" s="2"/>
-      <c r="I80" s="2"/>
+      <c r="C80" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D80" s="2">
+        <v>1</v>
+      </c>
+      <c r="E80" s="2">
+        <v>2</v>
+      </c>
+      <c r="F80" s="2">
+        <v>2</v>
+      </c>
+      <c r="G80" s="2">
+        <v>2</v>
+      </c>
+      <c r="H80" s="2">
+        <v>0</v>
+      </c>
+      <c r="I80" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="81" spans="1:9" ht="15">
       <c r="A81" s="2" t="s">
@@ -2016,13 +3114,27 @@
       <c r="B81" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="C81" s="2"/>
-      <c r="D81" s="2"/>
-      <c r="E81" s="2"/>
-      <c r="F81" s="2"/>
-      <c r="G81" s="2"/>
-      <c r="H81" s="2"/>
-      <c r="I81" s="2"/>
+      <c r="C81" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D81" s="2">
+        <v>1</v>
+      </c>
+      <c r="E81" s="2">
+        <v>1</v>
+      </c>
+      <c r="F81" s="2">
+        <v>1</v>
+      </c>
+      <c r="G81" s="2">
+        <v>1</v>
+      </c>
+      <c r="H81" s="2">
+        <v>0</v>
+      </c>
+      <c r="I81" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="82" spans="1:9" ht="15">
       <c r="A82" s="2" t="s">
@@ -2031,13 +3143,27 @@
       <c r="B82" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="C82" s="2"/>
-      <c r="D82" s="2"/>
-      <c r="E82" s="2"/>
-      <c r="F82" s="2"/>
-      <c r="G82" s="2"/>
-      <c r="H82" s="2"/>
-      <c r="I82" s="2"/>
+      <c r="C82" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D82" s="2">
+        <v>1</v>
+      </c>
+      <c r="E82" s="2">
+        <v>2</v>
+      </c>
+      <c r="F82" s="2">
+        <v>1</v>
+      </c>
+      <c r="G82" s="2">
+        <v>1</v>
+      </c>
+      <c r="H82" s="2">
+        <v>0</v>
+      </c>
+      <c r="I82" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="83" spans="1:9" ht="15">
       <c r="A83" s="2" t="s">
@@ -2046,13 +3172,27 @@
       <c r="B83" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C83" s="2"/>
-      <c r="D83" s="2"/>
-      <c r="E83" s="2"/>
-      <c r="F83" s="2"/>
-      <c r="G83" s="2"/>
-      <c r="H83" s="2"/>
-      <c r="I83" s="2"/>
+      <c r="C83" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D83" s="2">
+        <v>0</v>
+      </c>
+      <c r="E83" s="2">
+        <v>1</v>
+      </c>
+      <c r="F83" s="2">
+        <v>1</v>
+      </c>
+      <c r="G83" s="2">
+        <v>1</v>
+      </c>
+      <c r="H83" s="2">
+        <v>0</v>
+      </c>
+      <c r="I83" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="84" spans="1:9" ht="15">
       <c r="A84" s="2" t="s">
@@ -2061,13 +3201,27 @@
       <c r="B84" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C84" s="2"/>
-      <c r="D84" s="2"/>
-      <c r="E84" s="2"/>
-      <c r="F84" s="2"/>
-      <c r="G84" s="2"/>
-      <c r="H84" s="2"/>
-      <c r="I84" s="2"/>
+      <c r="C84" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D84" s="2">
+        <v>1</v>
+      </c>
+      <c r="E84" s="2">
+        <v>2</v>
+      </c>
+      <c r="F84" s="2">
+        <v>2</v>
+      </c>
+      <c r="G84" s="2">
+        <v>2</v>
+      </c>
+      <c r="H84" s="2">
+        <v>1</v>
+      </c>
+      <c r="I84" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="85" spans="1:9" ht="15">
       <c r="A85" s="2" t="s">
@@ -2076,13 +3230,27 @@
       <c r="B85" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="C85" s="2"/>
-      <c r="D85" s="2"/>
-      <c r="E85" s="2"/>
-      <c r="F85" s="2"/>
-      <c r="G85" s="2"/>
-      <c r="H85" s="2"/>
-      <c r="I85" s="2"/>
+      <c r="C85" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D85" s="2">
+        <v>1</v>
+      </c>
+      <c r="E85" s="2">
+        <v>2</v>
+      </c>
+      <c r="F85" s="2">
+        <v>2</v>
+      </c>
+      <c r="G85" s="2">
+        <v>2</v>
+      </c>
+      <c r="H85" s="2">
+        <v>1</v>
+      </c>
+      <c r="I85" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="86" spans="1:9" ht="15">
       <c r="A86" s="2" t="s">
@@ -2091,13 +3259,27 @@
       <c r="B86" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C86" s="2"/>
-      <c r="D86" s="2"/>
-      <c r="E86" s="2"/>
-      <c r="F86" s="2"/>
-      <c r="G86" s="2"/>
-      <c r="H86" s="2"/>
-      <c r="I86" s="2"/>
+      <c r="C86" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D86" s="2">
+        <v>1</v>
+      </c>
+      <c r="E86" s="2">
+        <v>2</v>
+      </c>
+      <c r="F86" s="2">
+        <v>2</v>
+      </c>
+      <c r="G86" s="2">
+        <v>2</v>
+      </c>
+      <c r="H86" s="2">
+        <v>1</v>
+      </c>
+      <c r="I86" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="87" spans="1:9" ht="15">
       <c r="A87" s="2" t="s">
@@ -2106,13 +3288,27 @@
       <c r="B87" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="C87" s="2"/>
-      <c r="D87" s="2"/>
-      <c r="E87" s="2"/>
-      <c r="F87" s="2"/>
-      <c r="G87" s="2"/>
-      <c r="H87" s="2"/>
-      <c r="I87" s="2"/>
+      <c r="C87" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D87" s="2">
+        <v>1</v>
+      </c>
+      <c r="E87" s="2">
+        <v>1</v>
+      </c>
+      <c r="F87" s="2">
+        <v>1</v>
+      </c>
+      <c r="G87" s="2">
+        <v>1</v>
+      </c>
+      <c r="H87" s="2">
+        <v>1</v>
+      </c>
+      <c r="I87" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="88" spans="1:9" ht="15">
       <c r="A88" s="2" t="s">
@@ -2121,13 +3317,27 @@
       <c r="B88" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="C88" s="2"/>
-      <c r="D88" s="2"/>
-      <c r="E88" s="2"/>
-      <c r="F88" s="2"/>
-      <c r="G88" s="2"/>
-      <c r="H88" s="2"/>
-      <c r="I88" s="2"/>
+      <c r="C88" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D88" s="2">
+        <v>2</v>
+      </c>
+      <c r="E88" s="2">
+        <v>1</v>
+      </c>
+      <c r="F88" s="2">
+        <v>1</v>
+      </c>
+      <c r="G88" s="2">
+        <v>1</v>
+      </c>
+      <c r="H88" s="2">
+        <v>2</v>
+      </c>
+      <c r="I88" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="89" spans="1:9" ht="15">
       <c r="A89" s="2" t="s">
@@ -2136,13 +3346,27 @@
       <c r="B89" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="C89" s="2"/>
-      <c r="D89" s="2"/>
-      <c r="E89" s="2"/>
-      <c r="F89" s="2"/>
-      <c r="G89" s="2"/>
-      <c r="H89" s="2"/>
-      <c r="I89" s="2"/>
+      <c r="C89" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D89" s="2">
+        <v>0</v>
+      </c>
+      <c r="E89" s="2">
+        <v>2</v>
+      </c>
+      <c r="F89" s="2">
+        <v>2</v>
+      </c>
+      <c r="G89" s="2">
+        <v>2</v>
+      </c>
+      <c r="H89" s="2">
+        <v>1</v>
+      </c>
+      <c r="I89" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="90" spans="1:9" ht="15">
       <c r="A90" s="2" t="s">
@@ -2151,13 +3375,27 @@
       <c r="B90" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C90" s="2"/>
-      <c r="D90" s="2"/>
-      <c r="E90" s="2"/>
-      <c r="F90" s="2"/>
-      <c r="G90" s="2"/>
-      <c r="H90" s="2"/>
-      <c r="I90" s="2"/>
+      <c r="C90" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D90" s="2">
+        <v>0</v>
+      </c>
+      <c r="E90" s="2">
+        <v>2</v>
+      </c>
+      <c r="F90" s="2">
+        <v>2</v>
+      </c>
+      <c r="G90" s="2">
+        <v>2</v>
+      </c>
+      <c r="H90" s="2">
+        <v>1</v>
+      </c>
+      <c r="I90" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="91" spans="1:9" ht="15">
       <c r="A91" s="2" t="s">
@@ -2166,16 +3404,42 @@
       <c r="B91" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C91" s="2"/>
-      <c r="D91" s="2"/>
-      <c r="E91" s="2"/>
-      <c r="F91" s="2"/>
-      <c r="G91" s="2"/>
-      <c r="H91" s="2"/>
-      <c r="I91" s="2"/>
+      <c r="C91" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D91" s="2">
+        <v>0</v>
+      </c>
+      <c r="E91" s="2">
+        <v>2</v>
+      </c>
+      <c r="F91" s="2">
+        <v>2</v>
+      </c>
+      <c r="G91" s="2">
+        <v>2</v>
+      </c>
+      <c r="H91" s="2">
+        <v>1</v>
+      </c>
+      <c r="I91" s="2">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="D2:I91">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
staged codes after addding up land price data
</commit_message>
<xml_diff>
--- a/poi/category-list-purpose-annotated.xlsx
+++ b/poi/category-list-purpose-annotated.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mario/github/google-poi-japan/poi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0B436CC-01D7-D74F-A7AA-802926125762}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93D499B9-F509-8F48-9D9E-45FBB11D0A3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14900" yWindow="-21100" windowWidth="19200" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -360,10 +360,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>acessibility family</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>tourist</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -393,6 +389,10 @@
   </si>
   <si>
     <t>learning/visiting</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>accessibility family</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -810,10 +810,10 @@
         <v>110</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="15">
@@ -824,7 +824,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D2" s="2">
         <v>2</v>
@@ -853,7 +853,7 @@
         <v>4</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D3" s="2">
         <v>2</v>
@@ -882,7 +882,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D4" s="2">
         <v>0</v>
@@ -911,7 +911,7 @@
         <v>6</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D5" s="2">
         <v>2</v>
@@ -940,7 +940,7 @@
         <v>7</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D6" s="2">
         <v>0</v>
@@ -969,7 +969,7 @@
         <v>9</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D7" s="2">
         <v>0</v>
@@ -998,7 +998,7 @@
         <v>10</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D8" s="2">
         <v>0</v>
@@ -1027,7 +1027,7 @@
         <v>11</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D9" s="2">
         <v>1</v>
@@ -1056,7 +1056,7 @@
         <v>12</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D10" s="2">
         <v>0</v>
@@ -1085,7 +1085,7 @@
         <v>13</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D11" s="2">
         <v>1</v>
@@ -1114,7 +1114,7 @@
         <v>14</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D12" s="2">
         <v>0</v>
@@ -1143,7 +1143,7 @@
         <v>15</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D13" s="2">
         <v>1</v>
@@ -1172,7 +1172,7 @@
         <v>17</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D14" s="2">
         <v>0</v>
@@ -1201,7 +1201,7 @@
         <v>18</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D15" s="2">
         <v>0</v>
@@ -1230,7 +1230,7 @@
         <v>19</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D16" s="2">
         <v>0</v>
@@ -1259,7 +1259,7 @@
         <v>20</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D17" s="2">
         <v>2</v>
@@ -1288,7 +1288,7 @@
         <v>21</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D18" s="2">
         <v>0</v>
@@ -1317,7 +1317,7 @@
         <v>22</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D19" s="2">
         <v>1</v>
@@ -1346,7 +1346,7 @@
         <v>23</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D20" s="2">
         <v>0</v>
@@ -1375,7 +1375,7 @@
         <v>24</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D21" s="2">
         <v>1</v>
@@ -1404,7 +1404,7 @@
         <v>25</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D22" s="2">
         <v>1</v>
@@ -1433,7 +1433,7 @@
         <v>26</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D23" s="2">
         <v>0</v>
@@ -1462,7 +1462,7 @@
         <v>28</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D24" s="2">
         <v>0</v>
@@ -1491,7 +1491,7 @@
         <v>29</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D25" s="2">
         <v>0</v>
@@ -1520,7 +1520,7 @@
         <v>30</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D26" s="2">
         <v>1</v>
@@ -1549,7 +1549,7 @@
         <v>31</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D27" s="2">
         <v>0</v>
@@ -1578,7 +1578,7 @@
         <v>32</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D28" s="2">
         <v>0</v>
@@ -1607,7 +1607,7 @@
         <v>33</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D29" s="2">
         <v>0</v>
@@ -1636,7 +1636,7 @@
         <v>34</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D30" s="2">
         <v>0</v>
@@ -1665,7 +1665,7 @@
         <v>36</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D31" s="2">
         <v>2</v>
@@ -1694,7 +1694,7 @@
         <v>37</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D32" s="2">
         <v>2</v>
@@ -1723,7 +1723,7 @@
         <v>38</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D33" s="2">
         <v>1</v>
@@ -1752,7 +1752,7 @@
         <v>39</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D34" s="2">
         <v>2</v>
@@ -1781,7 +1781,7 @@
         <v>41</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D35" s="2">
         <v>1</v>
@@ -1810,7 +1810,7 @@
         <v>42</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D36" s="2">
         <v>1</v>
@@ -1839,7 +1839,7 @@
         <v>43</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D37" s="2">
         <v>2</v>
@@ -1868,7 +1868,7 @@
         <v>44</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D38" s="2">
         <v>2</v>
@@ -1897,7 +1897,7 @@
         <v>45</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D39" s="2">
         <v>1</v>
@@ -1926,7 +1926,7 @@
         <v>46</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D40" s="2">
         <v>2</v>
@@ -1955,7 +1955,7 @@
         <v>47</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D41" s="2">
         <v>1</v>
@@ -1984,7 +1984,7 @@
         <v>49</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D42" s="2">
         <v>2</v>
@@ -2013,7 +2013,7 @@
         <v>50</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D43" s="2">
         <v>2</v>
@@ -2042,7 +2042,7 @@
         <v>51</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D44" s="2">
         <v>2</v>
@@ -2071,7 +2071,7 @@
         <v>52</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D45" s="2">
         <v>2</v>
@@ -2100,7 +2100,7 @@
         <v>53</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D46" s="2">
         <v>1</v>
@@ -2129,7 +2129,7 @@
         <v>54</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D47" s="2">
         <v>2</v>
@@ -2158,7 +2158,7 @@
         <v>55</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D48" s="2">
         <v>2</v>
@@ -2187,7 +2187,7 @@
         <v>56</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D49" s="2">
         <v>1</v>
@@ -2216,7 +2216,7 @@
         <v>58</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D50" s="2">
         <v>0</v>
@@ -2245,7 +2245,7 @@
         <v>59</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D51" s="2">
         <v>0</v>
@@ -2274,7 +2274,7 @@
         <v>60</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D52" s="2">
         <v>0</v>
@@ -2303,7 +2303,7 @@
         <v>61</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D53" s="2">
         <v>0</v>
@@ -2332,7 +2332,7 @@
         <v>63</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D54" s="2">
         <v>1</v>
@@ -2361,7 +2361,7 @@
         <v>64</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D55" s="2">
         <v>1</v>
@@ -2390,7 +2390,7 @@
         <v>65</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D56" s="2">
         <v>1</v>
@@ -2419,7 +2419,7 @@
         <v>66</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D57" s="2">
         <v>2</v>
@@ -2448,7 +2448,7 @@
         <v>67</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D58" s="2">
         <v>1</v>
@@ -2477,7 +2477,7 @@
         <v>68</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D59" s="2">
         <v>1</v>
@@ -2506,7 +2506,7 @@
         <v>70</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D60" s="2">
         <v>0</v>
@@ -2535,7 +2535,7 @@
         <v>71</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D61" s="2">
         <v>1</v>
@@ -2564,7 +2564,7 @@
         <v>72</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D62" s="2">
         <v>1</v>
@@ -2593,7 +2593,7 @@
         <v>73</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D63" s="2">
         <v>2</v>
@@ -2622,7 +2622,7 @@
         <v>74</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D64" s="2">
         <v>1</v>
@@ -2651,7 +2651,7 @@
         <v>75</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D65" s="2">
         <v>1</v>
@@ -2680,7 +2680,7 @@
         <v>76</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D66" s="2">
         <v>1</v>
@@ -2709,7 +2709,7 @@
         <v>77</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D67" s="2">
         <v>0</v>
@@ -2738,7 +2738,7 @@
         <v>79</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D68" s="2">
         <v>1</v>
@@ -2767,7 +2767,7 @@
         <v>80</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D69" s="2">
         <v>2</v>
@@ -2796,7 +2796,7 @@
         <v>81</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D70" s="2">
         <v>1</v>
@@ -2825,7 +2825,7 @@
         <v>82</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D71" s="2">
         <v>1</v>
@@ -2854,7 +2854,7 @@
         <v>83</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D72" s="2">
         <v>1</v>
@@ -2883,7 +2883,7 @@
         <v>84</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D73" s="2">
         <v>1</v>
@@ -2912,7 +2912,7 @@
         <v>85</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D74" s="2">
         <v>2</v>
@@ -2941,7 +2941,7 @@
         <v>86</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D75" s="2">
         <v>2</v>
@@ -2970,7 +2970,7 @@
         <v>88</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D76" s="2">
         <v>2</v>
@@ -2999,7 +2999,7 @@
         <v>89</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D77" s="2">
         <v>1</v>
@@ -3028,7 +3028,7 @@
         <v>90</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D78" s="2">
         <v>1</v>
@@ -3057,7 +3057,7 @@
         <v>92</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D79" s="2">
         <v>1</v>
@@ -3086,7 +3086,7 @@
         <v>93</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D80" s="2">
         <v>1</v>
@@ -3115,7 +3115,7 @@
         <v>94</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D81" s="2">
         <v>1</v>
@@ -3144,7 +3144,7 @@
         <v>95</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D82" s="2">
         <v>1</v>
@@ -3173,7 +3173,7 @@
         <v>96</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D83" s="2">
         <v>0</v>
@@ -3202,7 +3202,7 @@
         <v>97</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D84" s="2">
         <v>1</v>
@@ -3231,7 +3231,7 @@
         <v>98</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D85" s="2">
         <v>1</v>
@@ -3260,7 +3260,7 @@
         <v>99</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D86" s="2">
         <v>1</v>
@@ -3289,7 +3289,7 @@
         <v>100</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D87" s="2">
         <v>1</v>
@@ -3318,7 +3318,7 @@
         <v>101</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D88" s="2">
         <v>2</v>
@@ -3347,7 +3347,7 @@
         <v>103</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D89" s="2">
         <v>0</v>
@@ -3376,7 +3376,7 @@
         <v>104</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D90" s="2">
         <v>0</v>
@@ -3405,7 +3405,7 @@
         <v>105</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D91" s="2">
         <v>0</v>

</xml_diff>

<commit_message>
staged optimal results with remapping and trajectory data
</commit_message>
<xml_diff>
--- a/poi/category-list-purpose-annotated.xlsx
+++ b/poi/category-list-purpose-annotated.xlsx
@@ -1,21 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mario/github/google-poi-japan/poi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93D499B9-F509-8F48-9D9E-45FBB11D0A3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{082C1979-AE8D-6444-8380-4B4EA20273FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14900" yWindow="-21100" windowWidth="19200" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$C$1:$C$91</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -463,14 +479,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -777,8 +799,8 @@
   <dimension ref="A1:I91"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="2" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="22.5" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5" style="5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.33203125" bestFit="1" customWidth="1"/>
@@ -788,13 +810,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>106</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -817,13 +839,13 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="15">
-      <c r="A2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="2" t="s">
+      <c r="A2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D2" s="2">
@@ -846,13 +868,13 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="15">
-      <c r="A3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="s">
+      <c r="A3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D3" s="2">
@@ -875,13 +897,13 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="15">
-      <c r="A4" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="2" t="s">
+      <c r="A4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D4" s="2">
@@ -904,13 +926,13 @@
       </c>
     </row>
     <row r="5" spans="1:9" ht="15">
-      <c r="A5" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="2" t="s">
+      <c r="A5" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D5" s="2">
@@ -933,13 +955,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" ht="15">
-      <c r="A6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="2" t="s">
+      <c r="A6" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>113</v>
       </c>
       <c r="D6" s="2">
@@ -962,13 +984,13 @@
       </c>
     </row>
     <row r="7" spans="1:9" ht="15">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D7" s="2">
@@ -991,13 +1013,13 @@
       </c>
     </row>
     <row r="8" spans="1:9" ht="15">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D8" s="2">
@@ -1020,13 +1042,13 @@
       </c>
     </row>
     <row r="9" spans="1:9" ht="15">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D9" s="2">
@@ -1049,13 +1071,13 @@
       </c>
     </row>
     <row r="10" spans="1:9" ht="15">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D10" s="2">
@@ -1078,13 +1100,13 @@
       </c>
     </row>
     <row r="11" spans="1:9" ht="15">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D11" s="2">
@@ -1107,13 +1129,13 @@
       </c>
     </row>
     <row r="12" spans="1:9" ht="15">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D12" s="2">
@@ -1136,13 +1158,13 @@
       </c>
     </row>
     <row r="13" spans="1:9" ht="15">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D13" s="2">
@@ -1165,13 +1187,13 @@
       </c>
     </row>
     <row r="14" spans="1:9" ht="15">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D14" s="2">
@@ -1194,13 +1216,13 @@
       </c>
     </row>
     <row r="15" spans="1:9" ht="15">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D15" s="2">
@@ -1223,13 +1245,13 @@
       </c>
     </row>
     <row r="16" spans="1:9" ht="15">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D16" s="2">
@@ -1252,13 +1274,13 @@
       </c>
     </row>
     <row r="17" spans="1:9" ht="15">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D17" s="2">
@@ -1281,13 +1303,13 @@
       </c>
     </row>
     <row r="18" spans="1:9" ht="15">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D18" s="2">
@@ -1310,13 +1332,13 @@
       </c>
     </row>
     <row r="19" spans="1:9" ht="15">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D19" s="2">
@@ -1339,13 +1361,13 @@
       </c>
     </row>
     <row r="20" spans="1:9" ht="15">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D20" s="2">
@@ -1368,13 +1390,13 @@
       </c>
     </row>
     <row r="21" spans="1:9" ht="15">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D21" s="2">
@@ -1397,13 +1419,13 @@
       </c>
     </row>
     <row r="22" spans="1:9" ht="15">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D22" s="2">
@@ -1426,13 +1448,13 @@
       </c>
     </row>
     <row r="23" spans="1:9" ht="15">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D23" s="2">
@@ -1455,13 +1477,13 @@
       </c>
     </row>
     <row r="24" spans="1:9" ht="15">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="4" t="s">
         <v>117</v>
       </c>
       <c r="D24" s="2">
@@ -1484,13 +1506,13 @@
       </c>
     </row>
     <row r="25" spans="1:9" ht="15">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="4" t="s">
         <v>117</v>
       </c>
       <c r="D25" s="2">
@@ -1513,13 +1535,13 @@
       </c>
     </row>
     <row r="26" spans="1:9" ht="15">
-      <c r="A26" s="2" t="s">
+      <c r="A26" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="4" t="s">
         <v>117</v>
       </c>
       <c r="D26" s="2">
@@ -1542,13 +1564,13 @@
       </c>
     </row>
     <row r="27" spans="1:9" ht="15">
-      <c r="A27" s="2" t="s">
+      <c r="A27" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="4" t="s">
         <v>117</v>
       </c>
       <c r="D27" s="2">
@@ -1571,13 +1593,13 @@
       </c>
     </row>
     <row r="28" spans="1:9" ht="15">
-      <c r="A28" s="2" t="s">
+      <c r="A28" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C28" s="4" t="s">
         <v>117</v>
       </c>
       <c r="D28" s="2">
@@ -1600,13 +1622,13 @@
       </c>
     </row>
     <row r="29" spans="1:9" ht="15">
-      <c r="A29" s="2" t="s">
+      <c r="A29" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="C29" s="4" t="s">
         <v>117</v>
       </c>
       <c r="D29" s="2">
@@ -1629,13 +1651,13 @@
       </c>
     </row>
     <row r="30" spans="1:9" ht="15">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" s="4" t="s">
         <v>118</v>
       </c>
       <c r="D30" s="2">
@@ -1658,13 +1680,13 @@
       </c>
     </row>
     <row r="31" spans="1:9" ht="15">
-      <c r="A31" s="2" t="s">
+      <c r="A31" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C31" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D31" s="2">
@@ -1687,13 +1709,13 @@
       </c>
     </row>
     <row r="32" spans="1:9" ht="15">
-      <c r="A32" s="2" t="s">
+      <c r="A32" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D32" s="2">
@@ -1716,13 +1738,13 @@
       </c>
     </row>
     <row r="33" spans="1:9" ht="15">
-      <c r="A33" s="2" t="s">
+      <c r="A33" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="C33" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D33" s="2">
@@ -1745,13 +1767,13 @@
       </c>
     </row>
     <row r="34" spans="1:9" ht="15">
-      <c r="A34" s="2" t="s">
+      <c r="A34" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="C34" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D34" s="2">
@@ -1774,13 +1796,13 @@
       </c>
     </row>
     <row r="35" spans="1:9" ht="15">
-      <c r="A35" s="2" t="s">
+      <c r="A35" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="C35" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D35" s="2">
@@ -1803,13 +1825,13 @@
       </c>
     </row>
     <row r="36" spans="1:9" ht="15">
-      <c r="A36" s="2" t="s">
+      <c r="A36" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="C36" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D36" s="2">
@@ -1832,13 +1854,13 @@
       </c>
     </row>
     <row r="37" spans="1:9" ht="15">
-      <c r="A37" s="2" t="s">
+      <c r="A37" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B37" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="C37" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D37" s="2">
@@ -1861,13 +1883,13 @@
       </c>
     </row>
     <row r="38" spans="1:9" ht="15">
-      <c r="A38" s="2" t="s">
+      <c r="A38" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="C38" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D38" s="2">
@@ -1890,13 +1912,13 @@
       </c>
     </row>
     <row r="39" spans="1:9" ht="15">
-      <c r="A39" s="2" t="s">
+      <c r="A39" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="B39" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="C39" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D39" s="2">
@@ -1919,13 +1941,13 @@
       </c>
     </row>
     <row r="40" spans="1:9" ht="15">
-      <c r="A40" s="2" t="s">
+      <c r="A40" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="B40" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="C40" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D40" s="2">
@@ -1948,13 +1970,13 @@
       </c>
     </row>
     <row r="41" spans="1:9" ht="15">
-      <c r="A41" s="2" t="s">
+      <c r="A41" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="B41" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="C41" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D41" s="2">
@@ -1977,13 +1999,13 @@
       </c>
     </row>
     <row r="42" spans="1:9" ht="15">
-      <c r="A42" s="2" t="s">
+      <c r="A42" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C42" s="2" t="s">
+      <c r="C42" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D42" s="2">
@@ -2006,13 +2028,13 @@
       </c>
     </row>
     <row r="43" spans="1:9" ht="15">
-      <c r="A43" s="2" t="s">
+      <c r="A43" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B43" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C43" s="2" t="s">
+      <c r="C43" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D43" s="2">
@@ -2035,13 +2057,13 @@
       </c>
     </row>
     <row r="44" spans="1:9" ht="15">
-      <c r="A44" s="2" t="s">
+      <c r="A44" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B44" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="C44" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D44" s="2">
@@ -2064,13 +2086,13 @@
       </c>
     </row>
     <row r="45" spans="1:9" ht="15">
-      <c r="A45" s="2" t="s">
+      <c r="A45" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="B45" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C45" s="2" t="s">
+      <c r="C45" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D45" s="2">
@@ -2093,13 +2115,13 @@
       </c>
     </row>
     <row r="46" spans="1:9" ht="15">
-      <c r="A46" s="2" t="s">
+      <c r="A46" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B46" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C46" s="2" t="s">
+      <c r="C46" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D46" s="2">
@@ -2122,13 +2144,13 @@
       </c>
     </row>
     <row r="47" spans="1:9" ht="15">
-      <c r="A47" s="2" t="s">
+      <c r="A47" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="B47" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C47" s="2" t="s">
+      <c r="C47" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D47" s="2">
@@ -2151,13 +2173,13 @@
       </c>
     </row>
     <row r="48" spans="1:9" ht="15">
-      <c r="A48" s="2" t="s">
+      <c r="A48" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="B48" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C48" s="2" t="s">
+      <c r="C48" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D48" s="2">
@@ -2180,13 +2202,13 @@
       </c>
     </row>
     <row r="49" spans="1:9" ht="15">
-      <c r="A49" s="2" t="s">
+      <c r="A49" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="B49" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C49" s="2" t="s">
+      <c r="C49" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D49" s="2">
@@ -2209,13 +2231,13 @@
       </c>
     </row>
     <row r="50" spans="1:9" ht="15">
-      <c r="A50" s="2" t="s">
+      <c r="A50" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="B50" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C50" s="2" t="s">
+      <c r="C50" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D50" s="2">
@@ -2238,13 +2260,13 @@
       </c>
     </row>
     <row r="51" spans="1:9" ht="15">
-      <c r="A51" s="2" t="s">
+      <c r="A51" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="B51" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C51" s="2" t="s">
+      <c r="C51" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D51" s="2">
@@ -2267,13 +2289,13 @@
       </c>
     </row>
     <row r="52" spans="1:9" ht="15">
-      <c r="A52" s="2" t="s">
+      <c r="A52" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="B52" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C52" s="2" t="s">
+      <c r="C52" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D52" s="2">
@@ -2296,13 +2318,13 @@
       </c>
     </row>
     <row r="53" spans="1:9" ht="15">
-      <c r="A53" s="2" t="s">
+      <c r="A53" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="B53" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C53" s="2" t="s">
+      <c r="C53" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D53" s="2">
@@ -2325,13 +2347,13 @@
       </c>
     </row>
     <row r="54" spans="1:9" ht="15">
-      <c r="A54" s="2" t="s">
+      <c r="A54" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="B54" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C54" s="2" t="s">
+      <c r="C54" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D54" s="2">
@@ -2354,13 +2376,13 @@
       </c>
     </row>
     <row r="55" spans="1:9" ht="15">
-      <c r="A55" s="2" t="s">
+      <c r="A55" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="B55" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C55" s="2" t="s">
+      <c r="C55" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D55" s="2">
@@ -2383,13 +2405,13 @@
       </c>
     </row>
     <row r="56" spans="1:9" ht="15">
-      <c r="A56" s="2" t="s">
+      <c r="A56" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="B56" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C56" s="2" t="s">
+      <c r="C56" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D56" s="2">
@@ -2412,13 +2434,13 @@
       </c>
     </row>
     <row r="57" spans="1:9" ht="15">
-      <c r="A57" s="2" t="s">
+      <c r="A57" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B57" s="2" t="s">
+      <c r="B57" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="C57" s="2" t="s">
+      <c r="C57" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D57" s="2">
@@ -2441,13 +2463,13 @@
       </c>
     </row>
     <row r="58" spans="1:9" ht="15">
-      <c r="A58" s="2" t="s">
+      <c r="A58" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="B58" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="C58" s="2" t="s">
+      <c r="C58" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D58" s="2">
@@ -2470,13 +2492,13 @@
       </c>
     </row>
     <row r="59" spans="1:9" ht="15">
-      <c r="A59" s="2" t="s">
+      <c r="A59" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B59" s="2" t="s">
+      <c r="B59" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="C59" s="2" t="s">
+      <c r="C59" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D59" s="2">
@@ -2499,13 +2521,13 @@
       </c>
     </row>
     <row r="60" spans="1:9" ht="15">
-      <c r="A60" s="2" t="s">
+      <c r="A60" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="B60" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="C60" s="2" t="s">
+      <c r="C60" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D60" s="2">
@@ -2528,13 +2550,13 @@
       </c>
     </row>
     <row r="61" spans="1:9" ht="15">
-      <c r="A61" s="2" t="s">
+      <c r="A61" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B61" s="2" t="s">
+      <c r="B61" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="C61" s="2" t="s">
+      <c r="C61" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D61" s="2">
@@ -2557,13 +2579,13 @@
       </c>
     </row>
     <row r="62" spans="1:9" ht="15">
-      <c r="A62" s="2" t="s">
+      <c r="A62" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="B62" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C62" s="2" t="s">
+      <c r="C62" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D62" s="2">
@@ -2586,13 +2608,13 @@
       </c>
     </row>
     <row r="63" spans="1:9" ht="15">
-      <c r="A63" s="2" t="s">
+      <c r="A63" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B63" s="2" t="s">
+      <c r="B63" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C63" s="2" t="s">
+      <c r="C63" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D63" s="2">
@@ -2615,13 +2637,13 @@
       </c>
     </row>
     <row r="64" spans="1:9" ht="15">
-      <c r="A64" s="2" t="s">
+      <c r="A64" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B64" s="2" t="s">
+      <c r="B64" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="C64" s="2" t="s">
+      <c r="C64" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D64" s="2">
@@ -2644,13 +2666,13 @@
       </c>
     </row>
     <row r="65" spans="1:9" ht="15">
-      <c r="A65" s="2" t="s">
+      <c r="A65" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B65" s="2" t="s">
+      <c r="B65" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C65" s="2" t="s">
+      <c r="C65" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D65" s="2">
@@ -2673,13 +2695,13 @@
       </c>
     </row>
     <row r="66" spans="1:9" ht="15">
-      <c r="A66" s="2" t="s">
+      <c r="A66" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B66" s="2" t="s">
+      <c r="B66" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="C66" s="2" t="s">
+      <c r="C66" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D66" s="2">
@@ -2702,13 +2724,13 @@
       </c>
     </row>
     <row r="67" spans="1:9" ht="15">
-      <c r="A67" s="2" t="s">
+      <c r="A67" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B67" s="2" t="s">
+      <c r="B67" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C67" s="2" t="s">
+      <c r="C67" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D67" s="2">
@@ -2731,13 +2753,13 @@
       </c>
     </row>
     <row r="68" spans="1:9" ht="15">
-      <c r="A68" s="2" t="s">
+      <c r="A68" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B68" s="2" t="s">
+      <c r="B68" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C68" s="2" t="s">
+      <c r="C68" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D68" s="2">
@@ -2760,13 +2782,13 @@
       </c>
     </row>
     <row r="69" spans="1:9" ht="15">
-      <c r="A69" s="2" t="s">
+      <c r="A69" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B69" s="2" t="s">
+      <c r="B69" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C69" s="2" t="s">
+      <c r="C69" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D69" s="2">
@@ -2789,13 +2811,13 @@
       </c>
     </row>
     <row r="70" spans="1:9" ht="15">
-      <c r="A70" s="2" t="s">
+      <c r="A70" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B70" s="2" t="s">
+      <c r="B70" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C70" s="2" t="s">
+      <c r="C70" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D70" s="2">
@@ -2818,13 +2840,13 @@
       </c>
     </row>
     <row r="71" spans="1:9" ht="15">
-      <c r="A71" s="2" t="s">
+      <c r="A71" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B71" s="2" t="s">
+      <c r="B71" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="C71" s="2" t="s">
+      <c r="C71" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D71" s="2">
@@ -2847,13 +2869,13 @@
       </c>
     </row>
     <row r="72" spans="1:9" ht="15">
-      <c r="A72" s="2" t="s">
+      <c r="A72" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B72" s="2" t="s">
+      <c r="B72" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C72" s="2" t="s">
+      <c r="C72" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D72" s="2">
@@ -2876,13 +2898,13 @@
       </c>
     </row>
     <row r="73" spans="1:9" ht="15">
-      <c r="A73" s="2" t="s">
+      <c r="A73" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B73" s="2" t="s">
+      <c r="B73" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="C73" s="2" t="s">
+      <c r="C73" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D73" s="2">
@@ -2905,13 +2927,13 @@
       </c>
     </row>
     <row r="74" spans="1:9" ht="15">
-      <c r="A74" s="2" t="s">
+      <c r="A74" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B74" s="2" t="s">
+      <c r="B74" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="C74" s="2" t="s">
+      <c r="C74" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D74" s="2">
@@ -2934,13 +2956,13 @@
       </c>
     </row>
     <row r="75" spans="1:9" ht="15">
-      <c r="A75" s="2" t="s">
+      <c r="A75" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="B75" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="C75" s="2" t="s">
+      <c r="C75" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D75" s="2">
@@ -2963,13 +2985,13 @@
       </c>
     </row>
     <row r="76" spans="1:9" ht="15">
-      <c r="A76" s="2" t="s">
+      <c r="A76" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B76" s="2" t="s">
+      <c r="B76" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="C76" s="2" t="s">
+      <c r="C76" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D76" s="2">
@@ -2992,13 +3014,13 @@
       </c>
     </row>
     <row r="77" spans="1:9" ht="15">
-      <c r="A77" s="2" t="s">
+      <c r="A77" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B77" s="2" t="s">
+      <c r="B77" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="C77" s="2" t="s">
+      <c r="C77" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D77" s="2">
@@ -3021,13 +3043,13 @@
       </c>
     </row>
     <row r="78" spans="1:9" ht="15">
-      <c r="A78" s="2" t="s">
+      <c r="A78" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B78" s="2" t="s">
+      <c r="B78" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="C78" s="2" t="s">
+      <c r="C78" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D78" s="2">
@@ -3050,13 +3072,13 @@
       </c>
     </row>
     <row r="79" spans="1:9" ht="15">
-      <c r="A79" s="2" t="s">
+      <c r="A79" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="B79" s="2" t="s">
+      <c r="B79" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="C79" s="2" t="s">
+      <c r="C79" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D79" s="2">
@@ -3079,13 +3101,13 @@
       </c>
     </row>
     <row r="80" spans="1:9" ht="15">
-      <c r="A80" s="2" t="s">
+      <c r="A80" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="B80" s="2" t="s">
+      <c r="B80" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="C80" s="2" t="s">
+      <c r="C80" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D80" s="2">
@@ -3108,13 +3130,13 @@
       </c>
     </row>
     <row r="81" spans="1:9" ht="15">
-      <c r="A81" s="2" t="s">
+      <c r="A81" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="B81" s="2" t="s">
+      <c r="B81" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="C81" s="2" t="s">
+      <c r="C81" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D81" s="2">
@@ -3137,13 +3159,13 @@
       </c>
     </row>
     <row r="82" spans="1:9" ht="15">
-      <c r="A82" s="2" t="s">
+      <c r="A82" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="B82" s="2" t="s">
+      <c r="B82" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="C82" s="2" t="s">
+      <c r="C82" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D82" s="2">
@@ -3166,13 +3188,13 @@
       </c>
     </row>
     <row r="83" spans="1:9" ht="15">
-      <c r="A83" s="2" t="s">
+      <c r="A83" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="B83" s="2" t="s">
+      <c r="B83" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="C83" s="2" t="s">
+      <c r="C83" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D83" s="2">
@@ -3195,13 +3217,13 @@
       </c>
     </row>
     <row r="84" spans="1:9" ht="15">
-      <c r="A84" s="2" t="s">
+      <c r="A84" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="B84" s="2" t="s">
+      <c r="B84" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="C84" s="2" t="s">
+      <c r="C84" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D84" s="2">
@@ -3224,13 +3246,13 @@
       </c>
     </row>
     <row r="85" spans="1:9" ht="15">
-      <c r="A85" s="2" t="s">
+      <c r="A85" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="B85" s="2" t="s">
+      <c r="B85" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="C85" s="2" t="s">
+      <c r="C85" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D85" s="2">
@@ -3253,13 +3275,13 @@
       </c>
     </row>
     <row r="86" spans="1:9" ht="15">
-      <c r="A86" s="2" t="s">
+      <c r="A86" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="B86" s="2" t="s">
+      <c r="B86" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C86" s="2" t="s">
+      <c r="C86" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D86" s="2">
@@ -3282,13 +3304,13 @@
       </c>
     </row>
     <row r="87" spans="1:9" ht="15">
-      <c r="A87" s="2" t="s">
+      <c r="A87" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="B87" s="2" t="s">
+      <c r="B87" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="C87" s="2" t="s">
+      <c r="C87" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D87" s="2">
@@ -3311,13 +3333,13 @@
       </c>
     </row>
     <row r="88" spans="1:9" ht="15">
-      <c r="A88" s="2" t="s">
+      <c r="A88" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="B88" s="2" t="s">
+      <c r="B88" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="C88" s="2" t="s">
+      <c r="C88" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D88" s="2">
@@ -3340,13 +3362,13 @@
       </c>
     </row>
     <row r="89" spans="1:9" ht="15">
-      <c r="A89" s="2" t="s">
+      <c r="A89" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B89" s="2" t="s">
+      <c r="B89" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C89" s="2" t="s">
+      <c r="C89" s="4" t="s">
         <v>115</v>
       </c>
       <c r="D89" s="2">
@@ -3369,13 +3391,13 @@
       </c>
     </row>
     <row r="90" spans="1:9" ht="15">
-      <c r="A90" s="2" t="s">
+      <c r="A90" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B90" s="2" t="s">
+      <c r="B90" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="C90" s="2" t="s">
+      <c r="C90" s="4" t="s">
         <v>116</v>
       </c>
       <c r="D90" s="2">
@@ -3398,13 +3420,13 @@
       </c>
     </row>
     <row r="91" spans="1:9" ht="15">
-      <c r="A91" s="2" t="s">
+      <c r="A91" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B91" s="2" t="s">
+      <c r="B91" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="C91" s="2" t="s">
+      <c r="C91" s="4" t="s">
         <v>115</v>
       </c>
       <c r="D91" s="2">

</xml_diff>